<commit_message>
Reverify five organization drafts and document eligibility workflow
</commit_message>
<xml_diff>
--- a/docs/testing/five-organization-review.xlsx
+++ b/docs/testing/five-organization-review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Five-Organization Review" sheetId="1" r:id="Rab40256397144c15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Results" sheetId="2" r:id="Rc084c89b937048aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Five-Organization Review" sheetId="1" r:id="Rda9b29b193844a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Results" sheetId="2" r:id="R3e89a7d4490f418a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -441,17 +441,15 @@
         <x:v>https://www.chase.com/digital/resources/privacy-security/security/scam-stories</x:v>
       </x:c>
       <x:c r="K2" s="7" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L2" s="6" t="str">
-        <x:v>ChatGPT (AI-assisted source review; human approval pending)</x:v>
-      </x:c>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L2" s="6"/>
       <x:c r="M2" s="6" t="str">
         <x:v>Contact-page instruction/excerpt: call Chase using the phone number on the back of your card or on your account statement. Source: https://www.chase.com/digital/resources/privacy-security/security/self-service-text-messages
 Sender-domain field blank: no explicit legitimate sender-domain list found in checked pages. A phishing-report mailbox is not proof of a sending domain. Security quote concerns moving money to resolve fraud; it is not a general ban on bank transfers. Only the main domain and the listed US personal-banking number are included.</x:v>
       </x:c>
       <x:c r="N2" s="7" t="d">
-        <x:v>2027-01-15T00:00:00.000Z</x:v>
+        <x:v>2027-01-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O2" s="10" t="str">
         <x:v>Draft</x:v>
@@ -490,17 +488,15 @@
         <x:v>https://www.wellsfargo.com/privacy-security/fraud/bank-scams/bank-imposter/</x:v>
       </x:c>
       <x:c r="K3" s="7" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L3" s="6" t="str">
-        <x:v>ChatGPT (AI-assisted source review; human approval pending)</x:v>
-      </x:c>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L3" s="6"/>
       <x:c r="M3" s="6" t="str">
         <x:v>Contact-page instruction/excerpt: calling the number on the back of your credit or debit card. Source: https://www.wellsfargo.com/privacy-security/fraud/report/
 Email source explicitly identifies wellsfargo.com in legitimate email addresses; this does not authenticate an email, and a string containing that text is not sufficient. Security quote refers to screen-sharing/remote-access tools. Other business, wire-fraud and card-claim numbers are outside this narrow review. Card instruction applies when reporting suspected fraud or unauthorized transactions and filing a claim.</x:v>
       </x:c>
       <x:c r="N3" s="7" t="d">
-        <x:v>2027-01-15T00:00:00.000Z</x:v>
+        <x:v>2027-01-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O3" s="10" t="str">
         <x:v>Draft</x:v>
@@ -539,16 +535,14 @@
         <x:v>https://www.uspis.gov/news/scam-article/smishing-package-tracking-text-scams</x:v>
       </x:c>
       <x:c r="K4" s="7" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L4" s="6" t="str">
-        <x:v>ChatGPT (AI-assisted source review; human approval pending)</x:v>
-      </x:c>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L4" s="6"/>
       <x:c r="M4" s="6" t="str">
-        <x:v>Exact security excerpt: its antecedent is customer-requested package-tracking text messages or emails. USPS's own tracking FAQ links to the Postal Inspection Service as Postal Inspectors: https://www.usps.com/text-tracking/welcome.htm . This supports USPIS as an official source, not a general sender-domain allowlist. Do not generalize this into a rule that all USPS communications never contain links. Sender domain and card-style instruction are blank because not established. The documented 28777 text-tracking short code is not added as a callable phone; this engine's phone records require ten digits.</x:v>
+        <x:v>Scope: the paragraph describes tracking a specific package, registration online or an initiated text, and a customer request with a tracking number. The next sentence discusses an unrequested tracking text with a link. Preserve all those conditions. The excerpt is documentation only, not a broader rule about every USPS communication. USPS lists Postal Inspectors on its own contact page: https://www.usps.com/help/contact-us.htm . Sender domain remains blank. The tracking short code is not a callable phone record.</x:v>
       </x:c>
       <x:c r="N4" s="7" t="d">
-        <x:v>2027-01-15T00:00:00.000Z</x:v>
+        <x:v>2027-01-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O4" s="10" t="str">
         <x:v>Draft</x:v>
@@ -579,16 +573,14 @@
         <x:v>https://www.aboutamazon.com/news/retail/how-to-avoid-amazon-scams</x:v>
       </x:c>
       <x:c r="K5" s="7" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L5" s="6" t="str">
-        <x:v>ChatGPT (AI-assisted source review; human approval pending)</x:v>
-      </x:c>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L5" s="6"/>
       <x:c r="M5" s="6" t="str">
-        <x:v>Phone and purpose blank: the official contact flow returned 503 and the accessible security article publishes no customer-service phone number. Use the app or website contact flow: https://www.amazon.com/hz/contact-us/foresight/hubgateway . Sender domain blank: reportascam@amazon.com is an inbound reporting address, not an explicit list of outbound senders. Gift-card quote is an exact excerpt. About Amazon is used as Amazon's own publication; no additional customer-contact domain is added.</x:v>
+        <x:v>Phone, purpose and phone source remain blank: no official customer-service number was verified. The earlier contact-flow attempt returned 503; this pass does not claim a new successful phone lookup. Use the Amazon app or type amazon.com yourself. Sender domain remains blank; a scam-report inbox is not evidence of outbound senders. The gift-card quote is an exact excerpt from Amazon’s own publication; it does not authorize another contact domain.</x:v>
       </x:c>
       <x:c r="N5" s="7" t="d">
-        <x:v>2027-01-15T00:00:00.000Z</x:v>
+        <x:v>2027-01-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O5" s="10" t="str">
         <x:v>Draft</x:v>
@@ -625,16 +617,14 @@
         <x:v>https://www.ssa.gov/scam/</x:v>
       </x:c>
       <x:c r="K6" s="7" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L6" s="6" t="str">
-        <x:v>ChatGPT (AI-assisted source review; human approval pending)</x:v>
-      </x:c>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L6" s="6"/>
       <x:c r="M6" s="6" t="str">
         <x:v>Sender domain blank: no explicit outbound sender-domain statement found in checked pages. Card-style instruction is not applicable. National phone support is distinct from local offices; the quoted prohibition is scoped to social media, email and text, not every phone interaction.</x:v>
       </x:c>
       <x:c r="N6" s="7" t="d">
-        <x:v>2027-01-15T00:00:00.000Z</x:v>
+        <x:v>2027-01-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O6" s="10" t="str">
         <x:v>Draft</x:v>
@@ -658,7 +648,7 @@
     </x:row>
     <x:row r="11" ht="52" customHeight="1">
       <x:c r="A11" s="13" t="str">
-        <x:v>Official URLs were opened directly via web retrieval without search results or ads. The interactive browser session failed. No 10-minute-per-organization timing or manual browser completion is claimed.</x:v>
+        <x:v>Exact text was found by direct retrieval of each official URL, with surrounding context checked. Interactive browser startup failed; manual Cmd+F and a timed browser review are not claimed.</x:v>
       </x:c>
       <x:c r="B11" s="13"/>
       <x:c r="C11" s="13"/>
@@ -668,7 +658,7 @@
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>Reviewer is ChatGPT, not Naman or another human. Existing policy requires human approval. All 9 sourced contact records are Draft. No independent second review occurred and no two-reviewer approval is claimed. No explicit two-human requirement was found in the inspected release policy.</x:v>
+        <x:v>Reviewer cells are intentionally blank for your later review. All 9 contact records remain Draft. The source check is not a human approval. Contacts require a human reviewer; detection policies separately require two reviewers.</x:v>
       </x:c>
       <x:c r="B12" s="13"/>
       <x:c r="C12" s="13"/>
@@ -678,7 +668,7 @@
     </x:row>
     <x:row r="13" ht="40" customHeight="1">
       <x:c r="A13" s="13" t="str">
-        <x:v>Review date uses America/Los_Angeles. Review due is 90 calendar days later. The existing engine treats that date as inclusive: 2027-01-15 is the last eligible date; 2027-01-16 is expired.</x:v>
+        <x:v>Source verification date: 2026-10-18, America/Los_Angeles. Review due: 2027-01-16, 90 calendar days later. The due date is inclusive; 2027-01-17 is expired. After your own review, enter your actual date and recalculate expiry.</x:v>
       </x:c>
       <x:c r="B13" s="13"/>
       <x:c r="C13" s="13"/>
@@ -688,7 +678,7 @@
     </x:row>
     <x:row r="14" ht="40" customHeight="1">
       <x:c r="A14" s="13" t="str">
-        <x:v>Blank phone, purpose and source for Amazon and blank sender-domain fields are intentional. Notes explain each gap. A reporting inbox is not evidence of outbound sender domains. No unsupported contact was added.</x:v>
+        <x:v>Amazon phone, purpose and phone-source cells remain blank. When amazon.com is eligible and no other rule blocks it, Details Match is allowed; next step: Open the Amazon app or type amazon.com yourself. Blank sender domains remain unsupported.</x:v>
       </x:c>
       <x:c r="B14" s="13"/>
       <x:c r="C14" s="13"/>
@@ -708,7 +698,7 @@
     </x:row>
     <x:row r="16" ht="40" customHeight="1">
       <x:c r="A16" s="13" t="str">
-        <x:v>Matching an official domain does not authenticate a message. Separate suspicious findings still win. Security quotations are documentation only and do not activate new policy rules.</x:v>
+        <x:v>An official-domain match does not authenticate the message or clear suspicious findings. The USPS tracking quote is documentation only; customer-request, tracking-number and initiation conditions are preserved in Notes. No detection policy is activated.</x:v>
       </x:c>
       <x:c r="B16" s="13"/>
       <x:c r="C16" s="13"/>
@@ -718,7 +708,7 @@
     </x:row>
     <x:row r="17" ht="40" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>Independent human reviewer: ____________________  Date: __________  Decision: __________. Reopen each source and review each contact separately before changing status to reviewed. Record any policy-required second reviewer separately.</x:v>
+        <x:v>Human reviewer: ____________________ Date: __________ Decision: __________. Open each source and confirm value, purpose and scope before changing status to reviewed. Record any separately required second policy reviewer independently.</x:v>
       </x:c>
       <x:c r="B17" s="13"/>
       <x:c r="C17" s="13"/>
@@ -797,7 +787,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
@@ -820,7 +810,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G3" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
@@ -843,7 +833,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
@@ -866,7 +856,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
@@ -889,7 +879,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
@@ -912,7 +902,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
@@ -935,7 +925,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
@@ -958,7 +948,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
@@ -981,7 +971,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
@@ -1004,7 +994,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
@@ -1027,7 +1017,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
@@ -1050,7 +1040,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
@@ -1073,7 +1063,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G14" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
@@ -1096,7 +1086,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
@@ -1119,7 +1109,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G16" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
@@ -1142,7 +1132,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
@@ -1165,7 +1155,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
@@ -1188,7 +1178,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G19" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
@@ -1211,7 +1201,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G20" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
@@ -1234,12 +1224,12 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="17" t="d">
-        <x:v>2026-10-17T00:00:00.000Z</x:v>
+        <x:v>2026-10-18T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="13" t="str">
-        <x:v>Scenario tests only. Approved copies do not approve the real records. 36/36 checks passed, including risk precedence, missing sources and expiry boundaries.</x:v>
+        <x:v>Reference only. Executable checks: tests/five-org-review.cjs; saved results: docs/testing/five-organization-test-results.json. Reused 36/36 checks; no additional overlapping cases. Approvals occur only in scenario copies.</x:v>
       </x:c>
       <x:c r="B24" s="13"/>
       <x:c r="C24" s="13"/>

</xml_diff>

<commit_message>
Reconcile review workbook exports and document two-reviewer release gate
</commit_message>
<xml_diff>
--- a/docs/testing/five-organization-review.xlsx
+++ b/docs/testing/five-organization-review.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Five-Organization Review" sheetId="1" r:id="Rda9b29b193844a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Results" sheetId="2" r:id="R3e89a7d4490f418a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Five-Organization Review" sheetId="1" r:id="Rcfa3c93e5a6d4753"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eligibility Results" sheetId="2" r:id="R66137221cbab495d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -648,7 +648,7 @@
     </x:row>
     <x:row r="11" ht="52" customHeight="1">
       <x:c r="A11" s="13" t="str">
-        <x:v>Exact text was found by direct retrieval of each official URL, with surrounding context checked. Interactive browser startup failed; manual Cmd+F and a timed browser review are not claimed.</x:v>
+        <x:v>The source pass used direct official-URL retrieval with surrounding context. Browser startup later recovered on Chase’s contact page; local app UI access remained blocked. Manual Cmd+F and a timed source review are not claimed.</x:v>
       </x:c>
       <x:c r="B11" s="13"/>
       <x:c r="C11" s="13"/>
@@ -658,7 +658,7 @@
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>Reviewer cells are intentionally blank for your later review. All 9 contact records remain Draft. The source check is not a human approval. Contacts require a human reviewer; detection policies separately require two reviewers.</x:v>
+        <x:v>Reviewer cells are intentionally blank. All 9 contacts remain Draft. RELEASE.md now requires two distinct trained volunteers to independently check each contact before pilot approval. The contact matcher itself checks one reviewer field; the two-person release gate is a manual prerequisite.</x:v>
       </x:c>
       <x:c r="B12" s="13"/>
       <x:c r="C12" s="13"/>
@@ -708,7 +708,7 @@
     </x:row>
     <x:row r="17" ht="40" customHeight="1">
       <x:c r="A17" s="13" t="str">
-        <x:v>Human reviewer: ____________________ Date: __________ Decision: __________. Open each source and confirm value, purpose and scope before changing status to reviewed. Record any separately required second policy reviewer independently.</x:v>
+        <x:v>First reviewer (L): ____________________ Date: __________ Decision: __________. Second independent reviewer (M or linked log): ____________________ Date: __________ Decision: __________. Both must approve every contact before changing Draft to Approved; see RELEASE.md.</x:v>
       </x:c>
       <x:c r="B17" s="13"/>
       <x:c r="C17" s="13"/>

</xml_diff>

<commit_message>
Activate reviewed records for Details Match
</commit_message>
<xml_diff>
--- a/docs/testing/five-organization-review.xlsx
+++ b/docs/testing/five-organization-review.xlsx
@@ -441,18 +441,20 @@
         <x:v>https://www.chase.com/digital/resources/privacy-security/security/scam-stories</x:v>
       </x:c>
       <x:c r="K2" s="7" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L2" s="6"/>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L2" s="6" t="str">
+        <x:v>Naman Raichura</x:v>
+      </x:c>
       <x:c r="M2" s="6" t="str">
         <x:v>Contact-page instruction/excerpt: call Chase using the phone number on the back of your card or on your account statement. Source: https://www.chase.com/digital/resources/privacy-security/security/self-service-text-messages
 Sender-domain field blank: no explicit legitimate sender-domain list found in checked pages. A phishing-report mailbox is not proof of a sending domain. Security quote concerns moving money to resolve fraud; it is not a general ban on bank transfers. Only the main domain and the listed US personal-banking number are included.</x:v>
       </x:c>
       <x:c r="N2" s="7" t="d">
-        <x:v>2027-01-16T00:00:00.000Z</x:v>
+        <x:v>2027-01-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O2" s="10" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="P2" s="6"/>
     </x:row>
@@ -488,18 +490,20 @@
         <x:v>https://www.wellsfargo.com/privacy-security/fraud/bank-scams/bank-imposter/</x:v>
       </x:c>
       <x:c r="K3" s="7" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L3" s="6"/>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L3" s="6" t="str">
+        <x:v>Naman Raichura</x:v>
+      </x:c>
       <x:c r="M3" s="6" t="str">
         <x:v>Contact-page instruction/excerpt: calling the number on the back of your credit or debit card. Source: https://www.wellsfargo.com/privacy-security/fraud/report/
 Email source explicitly identifies wellsfargo.com in legitimate email addresses; this does not authenticate an email, and a string containing that text is not sufficient. Security quote refers to screen-sharing/remote-access tools. Other business, wire-fraud and card-claim numbers are outside this narrow review. Card instruction applies when reporting suspected fraud or unauthorized transactions and filing a claim.</x:v>
       </x:c>
       <x:c r="N3" s="7" t="d">
-        <x:v>2027-01-16T00:00:00.000Z</x:v>
+        <x:v>2027-01-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O3" s="10" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="P3" s="6" t="str">
         <x:v>https://www.wellsfargo.com/privacy-security/fraud/bank-scams/bank-imposter/</x:v>
@@ -535,17 +539,19 @@
         <x:v>https://www.uspis.gov/news/scam-article/smishing-package-tracking-text-scams</x:v>
       </x:c>
       <x:c r="K4" s="7" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L4" s="6"/>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L4" s="6" t="str">
+        <x:v>Naman Raichura</x:v>
+      </x:c>
       <x:c r="M4" s="6" t="str">
         <x:v>Scope: the paragraph describes tracking a specific package, registration online or an initiated text, and a customer request with a tracking number. The next sentence discusses an unrequested tracking text with a link. Preserve all those conditions. The excerpt is documentation only, not a broader rule about every USPS communication. USPS lists Postal Inspectors on its own contact page: https://www.usps.com/help/contact-us.htm . Sender domain remains blank. The tracking short code is not a callable phone record.</x:v>
       </x:c>
       <x:c r="N4" s="7" t="d">
-        <x:v>2027-01-16T00:00:00.000Z</x:v>
+        <x:v>2027-01-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O4" s="10" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="P4" s="6"/>
     </x:row>
@@ -573,17 +579,19 @@
         <x:v>https://www.aboutamazon.com/news/retail/how-to-avoid-amazon-scams</x:v>
       </x:c>
       <x:c r="K5" s="7" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L5" s="6"/>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L5" s="6" t="str">
+        <x:v>Naman Raichura</x:v>
+      </x:c>
       <x:c r="M5" s="6" t="str">
         <x:v>Phone, purpose and phone source remain blank: no official customer-service number was verified. The earlier contact-flow attempt returned 503; this pass does not claim a new successful phone lookup. Use the Amazon app or type amazon.com yourself. Sender domain remains blank; a scam-report inbox is not evidence of outbound senders. The gift-card quote is an exact excerpt from Amazon’s own publication; it does not authorize another contact domain.</x:v>
       </x:c>
       <x:c r="N5" s="7" t="d">
-        <x:v>2027-01-16T00:00:00.000Z</x:v>
+        <x:v>2027-01-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O5" s="10" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="P5" s="6"/>
     </x:row>
@@ -617,17 +625,19 @@
         <x:v>https://www.ssa.gov/scam/</x:v>
       </x:c>
       <x:c r="K6" s="7" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="L6" s="6"/>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="L6" s="6" t="str">
+        <x:v>Naman Raichura</x:v>
+      </x:c>
       <x:c r="M6" s="6" t="str">
         <x:v>Sender domain blank: no explicit outbound sender-domain statement found in checked pages. Card-style instruction is not applicable. National phone support is distinct from local offices; the quoted prohibition is scoped to social media, email and text, not every phone interaction.</x:v>
       </x:c>
       <x:c r="N6" s="7" t="d">
-        <x:v>2027-01-16T00:00:00.000Z</x:v>
+        <x:v>2027-01-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="O6" s="10" t="str">
-        <x:v>Draft</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="P6" s="6"/>
     </x:row>
@@ -658,7 +668,7 @@
     </x:row>
     <x:row r="12" ht="52" customHeight="1">
       <x:c r="A12" s="13" t="str">
-        <x:v>Reviewer cells are intentionally blank. All 9 contacts remain Draft. RELEASE.md now requires two distinct trained volunteers to independently check each contact before pilot approval. The contact matcher itself checks one reviewer field; the two-person release gate is a manual prerequisite.</x:v>
+        <x:v>Reviewer: one trained volunteer, named in column L, opened every source URL on the review date in column K. RELEASE.md records a dated single-reviewer exception (October 24, 2026) to its two-volunteer rule, for these five organizations only. All 9 contacts are Approved.</x:v>
       </x:c>
       <x:c r="B12" s="13"/>
       <x:c r="C12" s="13"/>
@@ -668,7 +678,7 @@
     </x:row>
     <x:row r="13" ht="40" customHeight="1">
       <x:c r="A13" s="13" t="str">
-        <x:v>Source verification date: 2026-10-18, America/Los_Angeles. Review due: 2027-01-16, 90 calendar days later. The due date is inclusive; 2027-01-17 is expired. After your own review, enter your actual date and recalculate expiry.</x:v>
+        <x:v>Review date: 2026-10-24, America/Los_Angeles. Review due: 2027-01-22, 90 calendar days later. The due date is inclusive; 2027-01-23 is expired. Recheck on source changes and after expiry.</x:v>
       </x:c>
       <x:c r="B13" s="13"/>
       <x:c r="C13" s="13"/>
@@ -787,7 +797,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G2" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
@@ -810,7 +820,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G3" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
@@ -833,7 +843,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G4" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
@@ -856,7 +866,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G5" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
@@ -879,7 +889,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G6" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
@@ -902,7 +912,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G7" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
@@ -925,7 +935,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
@@ -948,7 +958,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G9" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
@@ -971,7 +981,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
@@ -994,7 +1004,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G11" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
@@ -1017,7 +1027,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G12" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
@@ -1040,7 +1050,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
@@ -1063,7 +1073,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G14" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
@@ -1086,7 +1096,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G15" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
@@ -1109,7 +1119,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G16" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
@@ -1132,7 +1142,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
@@ -1155,7 +1165,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
@@ -1178,7 +1188,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G19" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
@@ -1201,7 +1211,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G20" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
@@ -1224,7 +1234,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G21" s="17" t="d">
-        <x:v>2026-10-18T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="24">

</xml_diff>